<commit_message>
added styles.css and map-handlers.js to www, added new data for OPM, Policia,DCR and CAVV, modify firt tab of SNMV to new layout and Maps in AVP for ne format for maps. Modify some renderMap functions, in process.
</commit_message>
<xml_diff>
--- a/data/Departamento_de_correccion_y_rehabilitacion/dcr_PSAJ.xlsx
+++ b/data/Departamento_de_correccion_y_rehabilitacion/dcr_PSAJ.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\orlan\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gnper\Documents\ViolenciaGeneroPR\data\Departamento_de_correccion_y_rehabilitacion\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{296E7E18-EB43-4274-A22C-90DCC747F83A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="10215" windowHeight="1500"/>
+    <workbookView xWindow="6936" yWindow="1860" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -64,7 +65,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -88,7 +89,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -96,12 +97,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -381,15 +400,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D13"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="26" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -403,7 +422,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>2024</v>
       </c>
@@ -413,11 +432,11 @@
       <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="1">
         <v>456</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2024</v>
       </c>
@@ -427,11 +446,11 @@
       <c r="C3" t="s">
         <v>4</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="1">
         <v>58</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>2025</v>
       </c>
@@ -441,11 +460,11 @@
       <c r="C4" t="s">
         <v>4</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="1">
         <v>395</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>2025</v>
       </c>
@@ -455,11 +474,11 @@
       <c r="C5" t="s">
         <v>4</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="1">
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>2026</v>
       </c>
@@ -469,11 +488,11 @@
       <c r="C6" t="s">
         <v>4</v>
       </c>
-      <c r="D6">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D6" s="1">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>2026</v>
       </c>
@@ -483,11 +502,11 @@
       <c r="C7" t="s">
         <v>4</v>
       </c>
-      <c r="D7">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D7" s="1">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>2024</v>
       </c>
@@ -497,11 +516,11 @@
       <c r="C8" t="s">
         <v>6</v>
       </c>
-      <c r="D8">
+      <c r="D8" s="1">
         <v>48</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>2024</v>
       </c>
@@ -511,11 +530,11 @@
       <c r="C9" t="s">
         <v>6</v>
       </c>
-      <c r="D9">
+      <c r="D9" s="1">
         <v>19</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>2025</v>
       </c>
@@ -525,11 +544,11 @@
       <c r="C10" t="s">
         <v>6</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="1">
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>2025</v>
       </c>
@@ -539,11 +558,11 @@
       <c r="C11" t="s">
         <v>6</v>
       </c>
-      <c r="D11">
+      <c r="D11" s="1">
         <v>14</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>2026</v>
       </c>
@@ -553,11 +572,11 @@
       <c r="C12" t="s">
         <v>6</v>
       </c>
-      <c r="D12">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D12" s="1">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>2026</v>
       </c>
@@ -567,7 +586,7 @@
       <c r="C13" t="s">
         <v>6</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="1">
         <v>14</v>
       </c>
     </row>

</xml_diff>